<commit_message>
feat: add comprehensive test reporting, form validation, and notification automation modules
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -9,12 +9,14 @@
     <sheet name="LoginCredentialsData" r:id="rId3" sheetId="1"/>
     <sheet name="TestCaseDefinitions" r:id="rId4" sheetId="2"/>
     <sheet name="TrainerReviewWorkflow" r:id="rId5" sheetId="3"/>
+    <sheet name="FormValidationWorkflow" r:id="rId6" sheetId="4"/>
+    <sheet name="NotificationWorkflow" r:id="rId7" sheetId="5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="154">
   <si>
     <t>Test_Type</t>
   </si>
@@ -290,6 +292,192 @@
   </si>
   <si>
     <t>REJECTED</t>
+  </si>
+  <si>
+    <t>User_Email</t>
+  </si>
+  <si>
+    <t>User_Password</t>
+  </si>
+  <si>
+    <t>Project_Title</t>
+  </si>
+  <si>
+    <t>Problem_Statement</t>
+  </si>
+  <si>
+    <t>Objectives</t>
+  </si>
+  <si>
+    <t>Tech_Stack</t>
+  </si>
+  <si>
+    <t>Doc_Link</t>
+  </si>
+  <si>
+    <t>Expected_Cohort_Title</t>
+  </si>
+  <si>
+    <t>Expected_Min_Alignment</t>
+  </si>
+  <si>
+    <t>PL-04</t>
+  </si>
+  <si>
+    <t>Open the new project submission page</t>
+  </si>
+  <si>
+    <t>The form opens for the Pod Lead and displays the active cohort criteria and the 70% minimum alignment requirement.</t>
+  </si>
+  <si>
+    <t>/submit</t>
+  </si>
+  <si>
+    <t>AI-Assisted Engineering</t>
+  </si>
+  <si>
+    <t>70%</t>
+  </si>
+  <si>
+    <t>PL-05</t>
+  </si>
+  <si>
+    <t>Submit the form with required information missing</t>
+  </si>
+  <si>
+    <t>Project title, problem statement, objectives and technology stack are validated. Submission is blocked until the required fields are completed; the documentation link remains optional.</t>
+  </si>
+  <si>
+    <t>Please complete all required fields.</t>
+  </si>
+  <si>
+    <t>PL-06</t>
+  </si>
+  <si>
+    <t>Submit a complete project idea</t>
+  </si>
+  <si>
+    <t>CloudAuto QA Platform</t>
+  </si>
+  <si>
+    <t>Software engineering teams face continuous delivery delays due to slow manual QA testing cycles. This platform automates regression workflows and provides real-time failure insights.</t>
+  </si>
+  <si>
+    <t>1. Automate 100% of critical core business workflows. 2. Integrate continuous feedback and defect detection. 3. Reduce manual regression effort by 60%.</t>
+  </si>
+  <si>
+    <t>Java, Spring Boot, Angular, REST API</t>
+  </si>
+  <si>
+    <t>https://github.com/projectlens/cloudauto-qa</t>
+  </si>
+  <si>
+    <t>The submission is saved, evaluation is initiated and the project appears in the Pod Lead's submissions list with its current status.</t>
+  </si>
+  <si>
+    <t>/submissions</t>
+  </si>
+  <si>
+    <t>PL-07</t>
+  </si>
+  <si>
+    <t>Verify a project evaluated below 70% alignment</t>
+  </si>
+  <si>
+    <t>The project is marked Needs Revision and the result clearly shows the score, analysis summary, matched criteria and missing criteria.</t>
+  </si>
+  <si>
+    <t>Expected_Alert_Keyword</t>
+  </si>
+  <si>
+    <t>Assigned_Pod</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_01</t>
+  </si>
+  <si>
+    <t>Open Notifications Page</t>
+  </si>
+  <si>
+    <t>Notifications page opens and displays a chronological list of recent updates with date and time.</t>
+  </si>
+  <si>
+    <t>/notifications</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>Pod Alpha</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_02</t>
+  </si>
+  <si>
+    <t>Low Score Alert (&lt; 70%)</t>
+  </si>
+  <si>
+    <t>Alert displays: Your project idea '[Idea Name]' needs improvement. Alignment score: [X]%. Please revise and reupload.</t>
+  </si>
+  <si>
+    <t>needs improvement. Alignment score:</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_03</t>
+  </si>
+  <si>
+    <t>High Score Alert (&gt;= 70%)</t>
+  </si>
+  <si>
+    <t>Alert displays: Your project idea '[Idea Name]' qualified for trainer review with an alignment score of [X]%.</t>
+  </si>
+  <si>
+    <t>qualified for trainer review with an alignment score of</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_04</t>
+  </si>
+  <si>
+    <t>Trainer Decision Alert</t>
+  </si>
+  <si>
+    <t>Alert displays trainer's decision, e.g., Trainer decision for '[Idea Name]': Approved.</t>
+  </si>
+  <si>
+    <t>Trainer decision for</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_05</t>
+  </si>
+  <si>
+    <t>Mark Notification as Read</t>
+  </si>
+  <si>
+    <t>Notification status updates to 'Read'.</t>
+  </si>
+  <si>
+    <t>Read</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_06</t>
+  </si>
+  <si>
+    <t>Refresh Notifications List</t>
+  </si>
+  <si>
+    <t>Page refreshes and fetches the latest notifications.</t>
+  </si>
+  <si>
+    <t>Refresh</t>
+  </si>
+  <si>
+    <t>TC_NOTIF_07</t>
+  </si>
+  <si>
+    <t>Pod Isolation Check</t>
+  </si>
+  <si>
+    <t>Pod Lead only sees notifications belonging to their assigned Pod and zero notifications from other pods.</t>
   </si>
 </sst>
 </file>
@@ -764,16 +952,204 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="5.63671875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="31.546875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="21.328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="15.34765625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="14.50390625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="13.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="62.9296875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="72.86328125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="14.8671875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="41.84765625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="20.2890625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.3046875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="19.7734375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="148.8125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="124.0546875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="29.703125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="37.40234375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="148.16015625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="28.98046875" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="19.6953125" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="21.69140625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -784,39 +1160,51 @@
         <v>25</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="I1" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="K1" t="s" s="0">
         <v>70</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>100</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>27</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>9</v>
@@ -828,27 +1216,39 @@
         <v>9</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>73</v>
+        <v>9</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>31</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>9</v>
@@ -857,97 +1257,332 @@
         <v>9</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>76</v>
+        <v>9</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>73</v>
+        <v>9</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>110</v>
+      </c>
+      <c r="L3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="M3" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>40</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>81</v>
+        <v>117</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="L4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="M4" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>43</v>
+        <v>120</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>83</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="I5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="K5" t="s" s="0">
         <v>86</v>
+      </c>
+      <c r="L5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="M5" t="s" s="0">
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="11.85546875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="21.69140625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="20.2890625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.3046875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="95.74609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="19.9765625" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="44.2578125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="12.12890625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>132</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>136</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>140</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>142</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>130</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>46</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>87</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>88</v>
+        <v>128</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>89</v>
+        <v>146</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="I6" t="s" s="0">
-        <v>91</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>152</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>153</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement Revise Submission module with Excel data-driven tests, POM, and standalone suite
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -11,12 +11,13 @@
     <sheet name="TrainerReviewWorkflow" r:id="rId5" sheetId="3"/>
     <sheet name="FormValidationWorkflow" r:id="rId6" sheetId="4"/>
     <sheet name="NotificationWorkflow" r:id="rId7" sheetId="5"/>
+    <sheet name="ReviseWorkflow" r:id="rId8" sheetId="6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="189">
   <si>
     <t>Test_Type</t>
   </si>
@@ -478,6 +479,111 @@
   </si>
   <si>
     <t>Pod Lead only sees notifications belonging to their assigned Pod and zero notifications from other pods.</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Test_Steps</t>
+  </si>
+  <si>
+    <t>Modified_Field</t>
+  </si>
+  <si>
+    <t>Modified_Value</t>
+  </si>
+  <si>
+    <t>Expected_Validation_Message</t>
+  </si>
+  <si>
+    <t>Verify Revise option is available</t>
+  </si>
+  <si>
+    <t>Pod Lead is logged in and has an existing submission.</t>
+  </si>
+  <si>
+    <t>1. Open Submissions. 2. Select the required submission. 3. Click Revise option.</t>
+  </si>
+  <si>
+    <t>Revise option should be available and the submission should open in editable mode.</t>
+  </si>
+  <si>
+    <t>/submit?revise=</t>
+  </si>
+  <si>
+    <t>Verify existing project details are displayed</t>
+  </si>
+  <si>
+    <t>Submission is opened in Revise mode.</t>
+  </si>
+  <si>
+    <t>1. Check Project Title. 2. Check Problem Statement, Objectives, Technology Stack and Documentation Link.</t>
+  </si>
+  <si>
+    <t>Previously entered project details should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify project details can be modified</t>
+  </si>
+  <si>
+    <t>Submission is in Revise mode.</t>
+  </si>
+  <si>
+    <t>1. Modify one or more project details. 2. Click Save/Continue.</t>
+  </si>
+  <si>
+    <t>Updated details should be accepted successfully.</t>
+  </si>
+  <si>
+    <t>problemStatement</t>
+  </si>
+  <si>
+    <t>Updated Problem Statement: Enterprise platform addressing delivery bottlenecks through automated QA and AI validation.</t>
+  </si>
+  <si>
+    <t>Verify mandatory field validation</t>
+  </si>
+  <si>
+    <t>1. Clear a mandatory field. 2. Click Re-upload/Submit.</t>
+  </si>
+  <si>
+    <t>Validation message should be displayed and submission should be prevented.</t>
+  </si>
+  <si>
+    <t>projectTitle</t>
+  </si>
+  <si>
+    <t>Verify revised project can be re-uploaded</t>
+  </si>
+  <si>
+    <t>Submission requires revision/re-upload.</t>
+  </si>
+  <si>
+    <t>1. Revise the project details. 2. Correct the required information. 3. Click Re-upload/Submit.</t>
+  </si>
+  <si>
+    <t>Revised project should be uploaded successfully and a confirmation message should be displayed.</t>
+  </si>
+  <si>
+    <t>objectives</t>
+  </si>
+  <si>
+    <t>1. Automate 100% of workflows. 2. Real-time telemetry. 3. Continuous defect prevention.</t>
+  </si>
+  <si>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>Verify updated submission and status after re-upload</t>
+  </si>
+  <si>
+    <t>Revised project has been successfully re-uploaded.</t>
+  </si>
+  <si>
+    <t>1. Open Submissions. 2. Open the revised submission. 3. Check project details and status.</t>
+  </si>
+  <si>
+    <t>Latest project details and updated submission status should be displayed correctly.</t>
   </si>
 </sst>
 </file>
@@ -1366,15 +1472,236 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>132</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>136</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>140</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>142</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>145</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>146</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>152</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>153</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="21.69140625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="5.63671875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="43.58984375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="20.2890625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.3046875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="95.74609375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="19.9765625" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="44.2578125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="12.12890625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="43.25390625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="86.30859375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="79.3671875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="19.9765625" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="16.15234375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="99.91796875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="28.98046875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1391,24 +1718,33 @@
         <v>93</v>
       </c>
       <c r="E1" t="s" s="0">
+        <v>154</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>155</v>
+      </c>
+      <c r="G1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="H1" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="G1" t="s" s="0">
-        <v>123</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>124</v>
+      <c r="I1" t="s" s="0">
+        <v>156</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>158</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>126</v>
+        <v>159</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>10</v>
@@ -1417,24 +1753,33 @@
         <v>11</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>129</v>
+        <v>162</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>130</v>
+        <v>163</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>131</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>132</v>
+        <v>164</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>10</v>
@@ -1443,24 +1788,33 @@
         <v>11</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>133</v>
+        <v>165</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>128</v>
+        <v>166</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>130</v>
+        <v>163</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>135</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>136</v>
+        <v>168</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>10</v>
@@ -1469,24 +1823,33 @@
         <v>11</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>137</v>
+        <v>169</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>128</v>
+        <v>170</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>130</v>
+        <v>163</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>139</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>140</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>10</v>
@@ -1495,24 +1858,33 @@
         <v>11</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>141</v>
+        <v>169</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>128</v>
+        <v>175</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>142</v>
+        <v>176</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>130</v>
+        <v>163</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="K5" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>143</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>10</v>
@@ -1521,24 +1893,33 @@
         <v>11</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>145</v>
+        <v>179</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>128</v>
+        <v>180</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>146</v>
+        <v>181</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>130</v>
+        <v>163</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>182</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>183</v>
+      </c>
+      <c r="K6" t="s" s="0">
+        <v>184</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>147</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>10</v>
@@ -1547,42 +1928,25 @@
         <v>11</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>149</v>
+        <v>186</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>128</v>
+        <v>187</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>151</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>152</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>153</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>128</v>
-      </c>
-      <c r="G8" t="s" s="0">
-        <v>130</v>
-      </c>
-      <c r="H8" t="s" s="0">
-        <v>130</v>
+        <v>119</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="J7" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="K7" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(fdu): implement Form Data Updation module (FDU_01 to FDU_10) with Excel DDT and 7-day scrum documentation
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -12,12 +12,13 @@
     <sheet name="FormValidationWorkflow" r:id="rId6" sheetId="4"/>
     <sheet name="NotificationWorkflow" r:id="rId7" sheetId="5"/>
     <sheet name="ReviseWorkflow" r:id="rId8" sheetId="6"/>
+    <sheet name="FormDataUpdationWorkflow" r:id="rId9" sheetId="7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="230">
   <si>
     <t>Test_Type</t>
   </si>
@@ -584,6 +585,129 @@
   </si>
   <si>
     <t>Latest project details and updated submission status should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Test_Case</t>
+  </si>
+  <si>
+    <t>Pod_Lead_Email</t>
+  </si>
+  <si>
+    <t>Pod_Lead_Password</t>
+  </si>
+  <si>
+    <t>Pod_Member_Email</t>
+  </si>
+  <si>
+    <t>Pod_Member_Password</t>
+  </si>
+  <si>
+    <t>FDU_01</t>
+  </si>
+  <si>
+    <t>Submit project details and verify data is stored</t>
+  </si>
+  <si>
+    <t>Project details are successfully saved in the system</t>
+  </si>
+  <si>
+    <t>OmniChannel AI Assistant</t>
+  </si>
+  <si>
+    <t>Customer service departments suffer from high response latencies and fragmented omnichannel conversation history.</t>
+  </si>
+  <si>
+    <t>1. Automate 80% repetitive queries. 2. Unified context across WhatsApp, Web and Email. 3. Real-time agent assist.</t>
+  </si>
+  <si>
+    <t>Java, Spring Boot, React, PostgreSQL</t>
+  </si>
+  <si>
+    <t>https://github.com/example/omnichannel-ai-specs</t>
+  </si>
+  <si>
+    <t>Innovex</t>
+  </si>
+  <si>
+    <t>FDU_02</t>
+  </si>
+  <si>
+    <t>Verify Project Title is updated after submission</t>
+  </si>
+  <si>
+    <t>Project Title is displayed correctly wherever the submission is viewed</t>
+  </si>
+  <si>
+    <t>FDU_03</t>
+  </si>
+  <si>
+    <t>Verify Problem Statement is updated after submission</t>
+  </si>
+  <si>
+    <t>Problem Statement is stored and displayed correctly</t>
+  </si>
+  <si>
+    <t>FDU_04</t>
+  </si>
+  <si>
+    <t>Verify Supporting Documentation Link is updated after submission</t>
+  </si>
+  <si>
+    <t>Documentation Link is stored and displayed correctly</t>
+  </si>
+  <si>
+    <t>FDU_05</t>
+  </si>
+  <si>
+    <t>Verify submitted data in Pod Lead view</t>
+  </si>
+  <si>
+    <t>Pod Lead can view the submitted details correctly</t>
+  </si>
+  <si>
+    <t>FDU_06</t>
+  </si>
+  <si>
+    <t>Verify submitted data in Pod Member view</t>
+  </si>
+  <si>
+    <t>Pod Member sees the same updated submission details</t>
+  </si>
+  <si>
+    <t>FDU_07</t>
+  </si>
+  <si>
+    <t>Verify submitted data in Trainer view</t>
+  </si>
+  <si>
+    <t>Trainer sees the same updated submission details</t>
+  </si>
+  <si>
+    <t>FDU_08</t>
+  </si>
+  <si>
+    <t>Verify data consistency across all roles</t>
+  </si>
+  <si>
+    <t>Data displayed in Pod Lead, Pod Member, and Trainer views should match exactly</t>
+  </si>
+  <si>
+    <t>FDU_09</t>
+  </si>
+  <si>
+    <t>Verify data persists after page refresh</t>
+  </si>
+  <si>
+    <t>Submitted data remains unchanged after refresh</t>
+  </si>
+  <si>
+    <t>FDU_10</t>
+  </si>
+  <si>
+    <t>Verify data persists after logout and login</t>
+  </si>
+  <si>
+    <t>Submitted data remains available after logging in again</t>
   </si>
 </sst>
 </file>
@@ -1952,4 +2076,548 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="7.30078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="54.12890625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="66.39453125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="20.2890625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="17.46875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="27.62890625" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="20.625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="21.328125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="15.34765625" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="21.5859375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="95.84375" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="92.90625" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="30.11328125" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="42.03515625" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="12.12890625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>192</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>193</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>95</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>194</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>196</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O2" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L3" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M3" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N3" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O3" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L4" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M4" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N4" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O4" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K5" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L5" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M5" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N5" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O5" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>213</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K6" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N6" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O6" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J7" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K7" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L7" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M7" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N7" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O7" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I8" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J8" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K8" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L8" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M8" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N8" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O8" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>222</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J9" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K9" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L9" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M9" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N9" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O9" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>226</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I10" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J10" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K10" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L10" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M10" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N10" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O10" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H11" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="I11" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="J11" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="K11" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="L11" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="M11" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="N11" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="O11" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>